<commit_message>
Trying other building intervention tables
</commit_message>
<xml_diff>
--- a/data/Interventions.xlsx
+++ b/data/Interventions.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8610e9849f4c2023/Documents/R/NCZ_Interventions/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9D330A69-1EC1-4EBA-8A15-7C1F53C4A18E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E6823D8-89A8-43A4-94A8-FB8A6C024009}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{9D330A69-1EC1-4EBA-8A15-7C1F53C4A18E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7457CA5-1C34-47A0-8B1E-56FA023C1F14}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{BBB8388B-3F78-4755-8EE7-BA9B37C5CC4B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" activeTab="1" xr2:uid="{BBB8388B-3F78-4755-8EE7-BA9B37C5CC4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="104">
   <si>
     <t>Building</t>
   </si>
@@ -198,19 +199,184 @@
   </si>
   <si>
     <t>Chiller EOL Replacement</t>
+  </si>
+  <si>
+    <t>One Federal</t>
+  </si>
+  <si>
+    <t>Retrocommissioning  (RCx)</t>
+  </si>
+  <si>
+    <t>Complete BMS commissioning </t>
+  </si>
+  <si>
+    <t> $ 9,000,000 </t>
+  </si>
+  <si>
+    <t>R&amp;M</t>
+  </si>
+  <si>
+    <t>  0.05 </t>
+  </si>
+  <si>
+    <t>  -   </t>
+  </si>
+  <si>
+    <t> $ -   </t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>RCx proposals </t>
+  </si>
+  <si>
+    <t>Optimal Start Stop </t>
+  </si>
+  <si>
+    <t>Sequence implementation in BMS</t>
+  </si>
+  <si>
+    <t> $ 65,000 </t>
+  </si>
+  <si>
+    <t>  0.01 </t>
+  </si>
+  <si>
+    <t> $ 5,000.00 </t>
+  </si>
+  <si>
+    <t>Controls Vendor</t>
+  </si>
+  <si>
+    <t>Chiller Plant Optimization</t>
+  </si>
+  <si>
+    <t>Analytic Program ontop of BMS</t>
+  </si>
+  <si>
+    <t> $ 8,000,000 </t>
+  </si>
+  <si>
+    <t>  0.04 </t>
+  </si>
+  <si>
+    <t>Optimun Energy </t>
+  </si>
+  <si>
+    <t> $ 200,000 </t>
+  </si>
+  <si>
+    <t>Schindler</t>
+  </si>
+  <si>
+    <t>DriveLine Retrofits </t>
+  </si>
+  <si>
+    <t>Electrificaiton</t>
+  </si>
+  <si>
+    <t>Electrification</t>
+  </si>
+  <si>
+    <t> $ 3,000,000 </t>
+  </si>
+  <si>
+    <t>  1.00 </t>
+  </si>
+  <si>
+    <t>York</t>
+  </si>
+  <si>
+    <t>New Electric Chillers </t>
+  </si>
+  <si>
+    <t>  3.00 </t>
+  </si>
+  <si>
+    <t>DHW to Point of Use </t>
+  </si>
+  <si>
+    <t> $ 380,000 </t>
+  </si>
+  <si>
+    <t>Eng</t>
+  </si>
+  <si>
+    <t>Façade air stopping </t>
+  </si>
+  <si>
+    <t> $ 2,000,000 </t>
+  </si>
+  <si>
+    <t>New High Efficiency Windows </t>
+  </si>
+  <si>
+    <t>New Windows tripple pane R6@30SHG</t>
+  </si>
+  <si>
+    <t> $ 22,958,333 </t>
+  </si>
+  <si>
+    <t>  0.06 </t>
+  </si>
+  <si>
+    <t>Spandrel and column insulation</t>
+  </si>
+  <si>
+    <t>Insulation at TI's</t>
+  </si>
+  <si>
+    <t> $ 1,000,000 </t>
+  </si>
+  <si>
+    <t>Electric Risistance Coils &amp; ASHP </t>
+  </si>
+  <si>
+    <t> $ 19,200,000 </t>
+  </si>
+  <si>
+    <t> $ 25,000.00 </t>
+  </si>
+  <si>
+    <t>Electric Risistance Coils &amp; ElectricHW Boiler </t>
+  </si>
+  <si>
+    <t> $ 5,200,000 </t>
+  </si>
+  <si>
+    <t>Electric Steam Boiler </t>
+  </si>
+  <si>
+    <t> $ 2,500,000 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -221,7 +387,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -229,12 +395,123 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF9A9A9A"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF9A9A9A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF9A9A9A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF6C6C6C"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF6C6C6C"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF6C6C6C"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF6C6C6C"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF6C6C6C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF6C6C6C"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF6C6C6C"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF6C6C6C"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF6C6C6C"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF6C6C6C"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,6 +978,9 @@
       <c r="M19">
         <v>2025</v>
       </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
       <c r="P19" t="s">
         <v>22</v>
       </c>
@@ -780,6 +1060,9 @@
       <c r="M21">
         <v>2025</v>
       </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
       <c r="P21" t="s">
         <v>22</v>
       </c>
@@ -818,6 +1101,9 @@
       <c r="M22">
         <v>2028</v>
       </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
       <c r="P22" t="s">
         <v>22</v>
       </c>
@@ -856,6 +1142,9 @@
       <c r="M23">
         <v>2025</v>
       </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
       <c r="P23" t="s">
         <v>22</v>
       </c>
@@ -894,6 +1183,9 @@
       <c r="M24">
         <v>2025</v>
       </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
       <c r="P24" t="s">
         <v>22</v>
       </c>
@@ -932,6 +1224,9 @@
       <c r="M25">
         <v>2029</v>
       </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
       <c r="P25" t="s">
         <v>22</v>
       </c>
@@ -970,6 +1265,9 @@
       <c r="M26">
         <v>2030</v>
       </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
       <c r="P26" t="s">
         <v>22</v>
       </c>
@@ -1008,6 +1306,9 @@
       <c r="M27">
         <v>2025</v>
       </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
       <c r="P27" t="s">
         <v>22</v>
       </c>
@@ -1046,6 +1347,9 @@
       <c r="M28">
         <v>2035</v>
       </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
       <c r="P28" t="s">
         <v>22</v>
       </c>
@@ -1084,8 +1388,724 @@
       <c r="M29">
         <v>2030</v>
       </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
       <c r="P29" t="s">
         <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11ECEFEA-BE52-4641-9A4D-3B7507A4E1C5}">
+  <dimension ref="A17:P30"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="7" width="14.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="17" spans="1:16" ht="45" customHeight="1">
+      <c r="A17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" t="s">
+        <v>4</v>
+      </c>
+      <c r="F17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" t="s">
+        <v>7</v>
+      </c>
+      <c r="I17" t="s">
+        <v>8</v>
+      </c>
+      <c r="J17" t="s">
+        <v>9</v>
+      </c>
+      <c r="K17" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" t="s">
+        <v>11</v>
+      </c>
+      <c r="M17" t="s">
+        <v>12</v>
+      </c>
+      <c r="N17" t="s">
+        <v>13</v>
+      </c>
+      <c r="O17" t="s">
+        <v>14</v>
+      </c>
+      <c r="P17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="46.5">
+      <c r="A18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="3">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L18" s="4">
+        <v>10</v>
+      </c>
+      <c r="M18" s="4">
+        <v>2025</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="34.5">
+      <c r="A19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="3">
+        <v>2</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="L19" s="4">
+        <v>12</v>
+      </c>
+      <c r="M19" s="4">
+        <v>2024</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="O19" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="46.5">
+      <c r="A20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="3">
+        <v>3</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20" s="4">
+        <v>12</v>
+      </c>
+      <c r="M20" s="4">
+        <v>2024</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P20" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="46.5">
+      <c r="A21" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="3">
+        <v>4</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="L21" s="4">
+        <v>25</v>
+      </c>
+      <c r="M21" s="4">
+        <v>2035</v>
+      </c>
+      <c r="N21" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O21" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P21" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="23.25">
+      <c r="A22" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="3">
+        <v>5</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22" s="4">
+        <v>-0.8</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L22" s="4">
+        <v>30</v>
+      </c>
+      <c r="M22" s="4">
+        <v>2028</v>
+      </c>
+      <c r="N22" s="7">
+        <v>-10000</v>
+      </c>
+      <c r="O22" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P22" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="23.25">
+      <c r="A23" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="3">
+        <v>5</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" s="4">
+        <v>-0.65</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="L23" s="4">
+        <v>30</v>
+      </c>
+      <c r="M23" s="4">
+        <v>2028</v>
+      </c>
+      <c r="N23" s="7">
+        <v>-25000</v>
+      </c>
+      <c r="O23" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P23" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="46.5">
+      <c r="A24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="3">
+        <v>6</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I24" s="4">
+        <v>-0.05</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L24" s="4">
+        <v>12</v>
+      </c>
+      <c r="M24" s="4">
+        <v>2024</v>
+      </c>
+      <c r="N24" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O24" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P24" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="34.5">
+      <c r="A25" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="3">
+        <v>7</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="L25" s="4">
+        <v>15</v>
+      </c>
+      <c r="M25" s="4">
+        <v>2023</v>
+      </c>
+      <c r="N25" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O25" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P25" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="46.5">
+      <c r="A26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="3">
+        <v>8</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="L26" s="4">
+        <v>10</v>
+      </c>
+      <c r="M26" s="4">
+        <v>2028</v>
+      </c>
+      <c r="N26" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O26" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P26" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="46.5">
+      <c r="A27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="3">
+        <v>9</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="L27" s="4">
+        <v>15</v>
+      </c>
+      <c r="M27" s="4">
+        <v>2024</v>
+      </c>
+      <c r="N27" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O27" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P27" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="34.5">
+      <c r="A28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="3">
+        <v>10</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I28" s="4">
+        <v>-1.5</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L28" s="4">
+        <v>40</v>
+      </c>
+      <c r="M28" s="4">
+        <v>2030</v>
+      </c>
+      <c r="N28" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="O28" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P28" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="57.75">
+      <c r="A29" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" s="3">
+        <v>10</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I29" s="4">
+        <v>-1</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L29" s="4">
+        <v>40</v>
+      </c>
+      <c r="M29" s="4">
+        <v>2030</v>
+      </c>
+      <c r="N29" s="7">
+        <v>-10000</v>
+      </c>
+      <c r="O29" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P29" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="23.25">
+      <c r="A30" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="3">
+        <v>10</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I30" s="4">
+        <v>-0.9</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L30" s="4">
+        <v>15</v>
+      </c>
+      <c r="M30" s="4">
+        <v>2026</v>
+      </c>
+      <c r="N30" s="7">
+        <v>-35000</v>
+      </c>
+      <c r="O30" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="P30" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>